<commit_message>
initial push to new repo
</commit_message>
<xml_diff>
--- a/BEDEL(2).xlsx
+++ b/BEDEL(2).xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="34">
   <si>
     <t>Description</t>
   </si>
@@ -122,12 +122,18 @@
   <si>
     <t>dimas</t>
   </si>
+  <si>
+    <t>Deduction</t>
+  </si>
+  <si>
+    <t>dimass</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -222,6 +228,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -231,7 +244,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -254,11 +267,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -524,6 +574,45 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -546,6 +635,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -857,40 +955,40 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.5703125" defaultRowHeight="24" customHeight="1"/>
   <sheetData>
     <row r="2" spans="2:8" ht="24" customHeight="1">
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="102" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="90">
+      <c r="C2" s="103">
         <f>SUM(D5:D14)</f>
         <v>700</v>
       </c>
-      <c r="D2" s="90"/>
-      <c r="F2" s="91">
+      <c r="D2" s="103"/>
+      <c r="F2" s="104">
         <v>9</v>
       </c>
-      <c r="G2" s="90">
+      <c r="G2" s="103">
         <f>SUM(H5:H35)</f>
         <v>2175</v>
       </c>
-      <c r="H2" s="90"/>
+      <c r="H2" s="103"/>
     </row>
     <row r="3" spans="2:8" ht="24" customHeight="1">
-      <c r="B3" s="89"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="F3" s="91"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
+      <c r="B3" s="102"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="F3" s="104"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
     </row>
     <row r="4" spans="2:8" ht="24" customHeight="1">
-      <c r="B4" s="89"/>
+      <c r="B4" s="102"/>
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="91"/>
+      <c r="F4" s="104"/>
       <c r="G4" s="8" t="s">
         <v>0</v>
       </c>
@@ -1333,20 +1431,20 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.5703125" defaultRowHeight="24" customHeight="1"/>
   <sheetData>
     <row r="2" spans="1:4" ht="24" customHeight="1">
-      <c r="B2" s="91"/>
-      <c r="C2" s="90">
+      <c r="B2" s="104"/>
+      <c r="C2" s="103">
         <f>SUM(D5:D31)</f>
         <v>2400</v>
       </c>
-      <c r="D2" s="90"/>
+      <c r="D2" s="103"/>
     </row>
     <row r="3" spans="1:4" ht="24" customHeight="1">
-      <c r="B3" s="91"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
+      <c r="B3" s="104"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
     </row>
     <row r="4" spans="1:4" ht="24" customHeight="1">
-      <c r="B4" s="91"/>
+      <c r="B4" s="104"/>
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
@@ -1558,58 +1656,58 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" ht="24" customHeight="1">
-      <c r="B2" s="92">
+      <c r="B2" s="105">
         <v>7</v>
       </c>
-      <c r="C2" s="93">
+      <c r="C2" s="106">
         <f>SUM(D5:D7)</f>
         <v>8500</v>
       </c>
-      <c r="D2" s="93"/>
-      <c r="F2" s="92">
+      <c r="D2" s="106"/>
+      <c r="F2" s="105">
         <v>8</v>
       </c>
-      <c r="G2" s="93">
+      <c r="G2" s="106">
         <f>SUM(H5:H7)</f>
         <v>8500</v>
       </c>
-      <c r="H2" s="93"/>
-      <c r="J2" s="92">
+      <c r="H2" s="106"/>
+      <c r="J2" s="105">
         <v>9</v>
       </c>
-      <c r="K2" s="93">
+      <c r="K2" s="106">
         <f>SUM(L5:L7)</f>
         <v>1500</v>
       </c>
-      <c r="L2" s="93"/>
+      <c r="L2" s="106"/>
     </row>
     <row r="3" spans="2:12" ht="24" customHeight="1">
-      <c r="B3" s="92"/>
-      <c r="C3" s="93"/>
-      <c r="D3" s="93"/>
-      <c r="F3" s="92"/>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93"/>
-      <c r="J3" s="92"/>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
+      <c r="B3" s="105"/>
+      <c r="C3" s="106"/>
+      <c r="D3" s="106"/>
+      <c r="F3" s="105"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="106"/>
+      <c r="J3" s="105"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="106"/>
     </row>
     <row r="4" spans="2:12" ht="24" customHeight="1">
-      <c r="B4" s="92"/>
+      <c r="B4" s="105"/>
       <c r="C4" s="9" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="92"/>
+      <c r="F4" s="105"/>
       <c r="G4" s="9" t="s">
         <v>0</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="J4" s="92"/>
+      <c r="J4" s="105"/>
       <c r="K4" s="9" t="s">
         <v>0</v>
       </c>
@@ -1680,56 +1778,56 @@
       <c r="F9" s="10"/>
     </row>
     <row r="10" spans="2:12" ht="24" customHeight="1">
-      <c r="B10" s="92">
+      <c r="B10" s="105">
         <v>10</v>
       </c>
-      <c r="C10" s="93">
+      <c r="C10" s="106">
         <f>SUM(D13:D39)</f>
         <v>8500</v>
       </c>
-      <c r="D10" s="93"/>
-      <c r="F10" s="92">
+      <c r="D10" s="106"/>
+      <c r="F10" s="105">
         <v>11</v>
       </c>
-      <c r="G10" s="93">
+      <c r="G10" s="106">
         <f>SUM(H13:H45)</f>
         <v>8500</v>
       </c>
-      <c r="H10" s="93"/>
-      <c r="J10" s="92"/>
-      <c r="K10" s="93">
+      <c r="H10" s="106"/>
+      <c r="J10" s="105"/>
+      <c r="K10" s="106">
         <f>SUM(L13:L44)</f>
         <v>4400</v>
       </c>
-      <c r="L10" s="93"/>
+      <c r="L10" s="106"/>
     </row>
     <row r="11" spans="2:12" ht="24" customHeight="1">
-      <c r="B11" s="92"/>
-      <c r="C11" s="93"/>
-      <c r="D11" s="93"/>
-      <c r="F11" s="92"/>
-      <c r="G11" s="93"/>
-      <c r="H11" s="93"/>
-      <c r="J11" s="92"/>
-      <c r="K11" s="93"/>
-      <c r="L11" s="93"/>
+      <c r="B11" s="105"/>
+      <c r="C11" s="106"/>
+      <c r="D11" s="106"/>
+      <c r="F11" s="105"/>
+      <c r="G11" s="106"/>
+      <c r="H11" s="106"/>
+      <c r="J11" s="105"/>
+      <c r="K11" s="106"/>
+      <c r="L11" s="106"/>
     </row>
     <row r="12" spans="2:12" ht="24" customHeight="1">
-      <c r="B12" s="92"/>
+      <c r="B12" s="105"/>
       <c r="C12" s="15" t="s">
         <v>0</v>
       </c>
       <c r="D12" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F12" s="92"/>
+      <c r="F12" s="105"/>
       <c r="G12" s="16" t="s">
         <v>0</v>
       </c>
       <c r="H12" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="J12" s="92"/>
+      <c r="J12" s="105"/>
       <c r="K12" s="19" t="s">
         <v>0</v>
       </c>
@@ -2333,155 +2431,155 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B2:AF61"/>
+  <dimension ref="B2:AF62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.5703125" defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="16384" width="17.5703125" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:32" ht="24" customHeight="1">
-      <c r="B2" s="95">
+      <c r="B2" s="108">
         <v>6</v>
       </c>
-      <c r="C2" s="94">
+      <c r="C2" s="107">
         <f>SUM(D5:D31)</f>
         <v>13000</v>
       </c>
-      <c r="D2" s="94"/>
-      <c r="F2" s="95">
+      <c r="D2" s="107"/>
+      <c r="F2" s="108">
         <v>7</v>
       </c>
-      <c r="G2" s="94">
+      <c r="G2" s="107">
         <f>SUM(H5:H32)</f>
         <v>13000</v>
       </c>
-      <c r="H2" s="94"/>
-      <c r="J2" s="95">
+      <c r="H2" s="107"/>
+      <c r="J2" s="108">
         <v>8</v>
       </c>
-      <c r="K2" s="94">
+      <c r="K2" s="107">
         <f>SUM(L5:L32)</f>
         <v>13000</v>
       </c>
-      <c r="L2" s="94"/>
-      <c r="N2" s="95">
+      <c r="L2" s="107"/>
+      <c r="N2" s="108">
         <v>9</v>
       </c>
-      <c r="O2" s="94">
+      <c r="O2" s="107">
         <f>SUM(P5:P8)</f>
         <v>13000</v>
       </c>
-      <c r="P2" s="94"/>
-      <c r="R2" s="95">
+      <c r="P2" s="107"/>
+      <c r="R2" s="108">
         <v>11</v>
       </c>
-      <c r="S2" s="94">
+      <c r="S2" s="107">
         <f>SUM(T5:T35)</f>
         <v>13000</v>
       </c>
-      <c r="T2" s="94"/>
-      <c r="V2" s="95">
-        <v>12</v>
-      </c>
-      <c r="W2" s="94">
+      <c r="T2" s="107"/>
+      <c r="V2" s="108">
+        <v>12</v>
+      </c>
+      <c r="W2" s="107">
         <f>SUM(X5:X35)</f>
         <v>16500</v>
       </c>
-      <c r="X2" s="94"/>
-      <c r="Z2" s="95">
+      <c r="X2" s="107"/>
+      <c r="Z2" s="108">
         <v>1</v>
       </c>
-      <c r="AA2" s="94">
+      <c r="AA2" s="107">
         <f>SUM(AB5:AB35)</f>
         <v>16500</v>
       </c>
-      <c r="AB2" s="94"/>
-      <c r="AD2" s="95">
+      <c r="AB2" s="107"/>
+      <c r="AD2" s="108">
         <v>2</v>
       </c>
-      <c r="AE2" s="94">
+      <c r="AE2" s="107">
         <f>SUM(AF6:AF37)</f>
         <v>16500</v>
       </c>
-      <c r="AF2" s="94"/>
+      <c r="AF2" s="107"/>
     </row>
     <row r="3" spans="2:32" ht="24" customHeight="1">
-      <c r="B3" s="95"/>
-      <c r="C3" s="94"/>
-      <c r="D3" s="94"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="94"/>
-      <c r="H3" s="94"/>
-      <c r="J3" s="95"/>
-      <c r="K3" s="94"/>
-      <c r="L3" s="94"/>
-      <c r="N3" s="95"/>
-      <c r="O3" s="94"/>
-      <c r="P3" s="94"/>
-      <c r="R3" s="95"/>
-      <c r="S3" s="94"/>
-      <c r="T3" s="94"/>
-      <c r="V3" s="95"/>
-      <c r="W3" s="94"/>
-      <c r="X3" s="94"/>
-      <c r="Z3" s="95"/>
-      <c r="AA3" s="94"/>
-      <c r="AB3" s="94"/>
-      <c r="AD3" s="95"/>
-      <c r="AE3" s="94"/>
-      <c r="AF3" s="94"/>
+      <c r="B3" s="108"/>
+      <c r="C3" s="107"/>
+      <c r="D3" s="107"/>
+      <c r="F3" s="108"/>
+      <c r="G3" s="107"/>
+      <c r="H3" s="107"/>
+      <c r="J3" s="108"/>
+      <c r="K3" s="107"/>
+      <c r="L3" s="107"/>
+      <c r="N3" s="108"/>
+      <c r="O3" s="107"/>
+      <c r="P3" s="107"/>
+      <c r="R3" s="108"/>
+      <c r="S3" s="107"/>
+      <c r="T3" s="107"/>
+      <c r="V3" s="108"/>
+      <c r="W3" s="107"/>
+      <c r="X3" s="107"/>
+      <c r="Z3" s="108"/>
+      <c r="AA3" s="107"/>
+      <c r="AB3" s="107"/>
+      <c r="AD3" s="108"/>
+      <c r="AE3" s="107"/>
+      <c r="AF3" s="107"/>
     </row>
     <row r="4" spans="2:32" ht="24" customHeight="1">
-      <c r="B4" s="95"/>
+      <c r="B4" s="108"/>
       <c r="C4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="95"/>
+      <c r="F4" s="108"/>
       <c r="G4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="J4" s="95"/>
+      <c r="J4" s="108"/>
       <c r="K4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="N4" s="95"/>
+      <c r="N4" s="108"/>
       <c r="O4" s="6" t="s">
         <v>0</v>
       </c>
       <c r="P4" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="R4" s="95"/>
+      <c r="R4" s="108"/>
       <c r="S4" s="18" t="s">
         <v>0</v>
       </c>
       <c r="T4" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="V4" s="95"/>
+      <c r="V4" s="108"/>
       <c r="W4" s="20" t="s">
         <v>0</v>
       </c>
       <c r="X4" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="Z4" s="95"/>
+      <c r="Z4" s="108"/>
       <c r="AA4" s="23" t="s">
         <v>0</v>
       </c>
       <c r="AB4" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="AD4" s="95"/>
+      <c r="AD4" s="108"/>
       <c r="AE4" s="41" t="s">
         <v>0</v>
       </c>
@@ -2919,14 +3017,14 @@
       <c r="L11" s="2">
         <v>100</v>
       </c>
-      <c r="N11" s="95">
+      <c r="N11" s="108">
         <v>10</v>
       </c>
-      <c r="O11" s="94">
+      <c r="O11" s="107">
         <f>SUM(P14:P44)</f>
         <v>13000</v>
       </c>
-      <c r="P11" s="94"/>
+      <c r="P11" s="107"/>
       <c r="R11" s="1">
         <v>45962</v>
       </c>
@@ -2989,9 +3087,9 @@
       <c r="L12" s="2">
         <v>100</v>
       </c>
-      <c r="N12" s="95"/>
-      <c r="O12" s="94"/>
-      <c r="P12" s="94"/>
+      <c r="N12" s="108"/>
+      <c r="O12" s="107"/>
+      <c r="P12" s="107"/>
       <c r="R12" s="1">
         <v>45963</v>
       </c>
@@ -3054,7 +3152,7 @@
       <c r="L13" s="2">
         <v>100</v>
       </c>
-      <c r="N13" s="95"/>
+      <c r="N13" s="108"/>
       <c r="O13" s="14" t="s">
         <v>0</v>
       </c>
@@ -4494,20 +4592,28 @@
       </c>
     </row>
     <row r="35" spans="2:32" ht="24" customHeight="1">
-      <c r="B35" s="95"/>
-      <c r="C35" s="94">
+      <c r="B35" s="108"/>
+      <c r="C35" s="107">
         <f>SUM(D38:D70)</f>
         <v>2750</v>
       </c>
-      <c r="D35" s="94"/>
-      <c r="F35" s="95">
+      <c r="D35" s="107"/>
+      <c r="F35" s="108">
         <v>3</v>
       </c>
-      <c r="G35" s="94">
+      <c r="G35" s="107">
         <f>SUM(H38:H73)</f>
-        <v>8600</v>
-      </c>
-      <c r="H35" s="94"/>
+        <v>16500</v>
+      </c>
+      <c r="H35" s="107"/>
+      <c r="J35" s="108">
+        <v>4</v>
+      </c>
+      <c r="K35" s="107">
+        <f>SUM(L38:L73)</f>
+        <v>850</v>
+      </c>
+      <c r="L35" s="107"/>
       <c r="N35" s="1">
         <v>45946</v>
       </c>
@@ -4528,12 +4634,15 @@
       </c>
     </row>
     <row r="36" spans="2:32" ht="24" customHeight="1">
-      <c r="B36" s="95"/>
-      <c r="C36" s="94"/>
-      <c r="D36" s="94"/>
-      <c r="F36" s="95"/>
-      <c r="G36" s="94"/>
-      <c r="H36" s="94"/>
+      <c r="B36" s="108"/>
+      <c r="C36" s="107"/>
+      <c r="D36" s="107"/>
+      <c r="F36" s="108"/>
+      <c r="G36" s="107"/>
+      <c r="H36" s="107"/>
+      <c r="J36" s="108"/>
+      <c r="K36" s="107"/>
+      <c r="L36" s="107"/>
       <c r="N36" s="1">
         <v>45947</v>
       </c>
@@ -4554,18 +4663,25 @@
       </c>
     </row>
     <row r="37" spans="2:32" ht="24" customHeight="1">
-      <c r="B37" s="95"/>
+      <c r="B37" s="108"/>
       <c r="C37" s="66" t="s">
         <v>0</v>
       </c>
       <c r="D37" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="F37" s="95"/>
+      <c r="F37" s="108"/>
       <c r="G37" s="73" t="s">
         <v>0</v>
       </c>
       <c r="H37" s="73" t="s">
+        <v>1</v>
+      </c>
+      <c r="J37" s="108"/>
+      <c r="K37" s="94" t="s">
+        <v>0</v>
+      </c>
+      <c r="L37" s="94" t="s">
         <v>1</v>
       </c>
       <c r="N37" s="1">
@@ -4606,6 +4722,15 @@
       <c r="H38" s="2" t="s">
         <v>28</v>
       </c>
+      <c r="J38" s="97">
+        <v>46114</v>
+      </c>
+      <c r="K38" s="98" t="s">
+        <v>5</v>
+      </c>
+      <c r="L38" s="2">
+        <v>100</v>
+      </c>
       <c r="N38" s="1">
         <v>45949</v>
       </c>
@@ -4635,6 +4760,15 @@
       <c r="H39" s="2" t="s">
         <v>28</v>
       </c>
+      <c r="J39" s="97">
+        <v>46115</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L39" s="2">
+        <v>150</v>
+      </c>
       <c r="N39" s="1">
         <v>45950</v>
       </c>
@@ -4664,6 +4798,15 @@
       <c r="H40" s="2">
         <v>200</v>
       </c>
+      <c r="J40" s="97">
+        <v>46116</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="N40" s="1">
         <v>45951</v>
       </c>
@@ -4693,6 +4836,15 @@
       <c r="H41" s="2">
         <v>100</v>
       </c>
+      <c r="J41" s="97">
+        <v>46117</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="L41" s="2">
+        <v>300</v>
+      </c>
       <c r="N41" s="1">
         <v>45952</v>
       </c>
@@ -4722,6 +4874,15 @@
       <c r="H42" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="J42" s="97">
+        <v>46118</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L42" s="2">
+        <v>100</v>
+      </c>
       <c r="N42" s="1">
         <v>45953</v>
       </c>
@@ -4748,6 +4909,12 @@
       <c r="H43" s="2">
         <v>100</v>
       </c>
+      <c r="J43" s="97">
+        <v>46119</v>
+      </c>
+      <c r="L43" s="2">
+        <v>100</v>
+      </c>
       <c r="N43" s="1">
         <v>45954</v>
       </c>
@@ -4768,6 +4935,12 @@
       <c r="H44" s="2">
         <v>100</v>
       </c>
+      <c r="J44" s="97">
+        <v>46120</v>
+      </c>
+      <c r="L44" s="2">
+        <v>100</v>
+      </c>
       <c r="N44" s="1">
         <v>45955</v>
       </c>
@@ -4965,8 +5138,19 @@
         <v>1200</v>
       </c>
     </row>
+    <row r="62" spans="6:8" ht="24" customHeight="1">
+      <c r="F62" s="1">
+        <v>46114</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H62" s="2">
+        <v>7900</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="24">
     <mergeCell ref="AE2:AF3"/>
     <mergeCell ref="K2:L3"/>
     <mergeCell ref="R2:R4"/>
@@ -4989,6 +5173,8 @@
     <mergeCell ref="N11:N13"/>
     <mergeCell ref="F35:F37"/>
     <mergeCell ref="G35:H36"/>
+    <mergeCell ref="J35:J37"/>
+    <mergeCell ref="K35:L36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5004,40 +5190,40 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="24" customHeight="1">
-      <c r="B2" s="96">
+      <c r="B2" s="109">
         <v>11</v>
       </c>
-      <c r="C2" s="90">
+      <c r="C2" s="103">
         <f>SUM(D5:D31)</f>
         <v>2750</v>
       </c>
-      <c r="D2" s="90"/>
-      <c r="F2" s="96">
-        <v>12</v>
-      </c>
-      <c r="G2" s="90">
+      <c r="D2" s="103"/>
+      <c r="F2" s="109">
+        <v>12</v>
+      </c>
+      <c r="G2" s="103">
         <f>SUM(H5:H29)</f>
         <v>15470</v>
       </c>
-      <c r="H2" s="90"/>
+      <c r="H2" s="103"/>
     </row>
     <row r="3" spans="2:8" ht="24" customHeight="1">
-      <c r="B3" s="96"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
+      <c r="B3" s="109"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="F3" s="109"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
     </row>
     <row r="4" spans="2:8" ht="24" customHeight="1">
-      <c r="B4" s="96"/>
+      <c r="B4" s="109"/>
       <c r="C4" s="21" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="96"/>
+      <c r="F4" s="109"/>
       <c r="G4" s="21" t="s">
         <v>0</v>
       </c>
@@ -5402,91 +5588,110 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B2:Q38"/>
+  <dimension ref="B2:T38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.5703125" defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="16384" width="17.5703125" style="25"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" ht="24" customHeight="1">
-      <c r="B2" s="96">
-        <v>12</v>
-      </c>
-      <c r="C2" s="90">
+    <row r="2" spans="2:20" ht="24" customHeight="1">
+      <c r="B2" s="109">
+        <v>12</v>
+      </c>
+      <c r="C2" s="103">
         <f>SUM(D6:D39)</f>
         <v>8500</v>
       </c>
-      <c r="D2" s="90"/>
-      <c r="F2" s="96">
+      <c r="D2" s="103"/>
+      <c r="F2" s="109">
         <v>1</v>
       </c>
-      <c r="G2" s="90">
+      <c r="G2" s="103">
         <f>SUM(H5:H39)</f>
         <v>10500</v>
       </c>
-      <c r="H2" s="90"/>
-      <c r="J2" s="96">
+      <c r="H2" s="103"/>
+      <c r="J2" s="109">
         <v>2</v>
       </c>
-      <c r="K2" s="90">
+      <c r="K2" s="103">
         <f>SUM(L5:L39)</f>
         <v>10150</v>
       </c>
-      <c r="L2" s="90"/>
-      <c r="N2" s="96">
+      <c r="L2" s="103"/>
+      <c r="N2" s="110">
         <v>3</v>
       </c>
-      <c r="O2" s="90">
+      <c r="O2" s="103">
         <f>SUM(P5:P39)</f>
-        <v>2000</v>
-      </c>
-      <c r="P2" s="90"/>
-    </row>
-    <row r="3" spans="2:16" ht="24" customHeight="1">
-      <c r="B3" s="96"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="90"/>
-      <c r="L3" s="90"/>
-      <c r="N3" s="96"/>
-      <c r="O3" s="90"/>
-      <c r="P3" s="90"/>
-    </row>
-    <row r="4" spans="2:16" ht="24" customHeight="1">
-      <c r="B4" s="96"/>
+        <v>10500</v>
+      </c>
+      <c r="P2" s="103"/>
+      <c r="R2" s="110">
+        <v>4</v>
+      </c>
+      <c r="S2" s="103">
+        <f>SUM(T5:T39)</f>
+        <v>1350</v>
+      </c>
+      <c r="T2" s="103"/>
+    </row>
+    <row r="3" spans="2:20" ht="24" customHeight="1">
+      <c r="B3" s="109"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="F3" s="109"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
+      <c r="J3" s="109"/>
+      <c r="K3" s="103"/>
+      <c r="L3" s="103"/>
+      <c r="N3" s="111"/>
+      <c r="O3" s="103"/>
+      <c r="P3" s="103"/>
+      <c r="R3" s="111"/>
+      <c r="S3" s="103"/>
+      <c r="T3" s="103"/>
+    </row>
+    <row r="4" spans="2:20" ht="24" customHeight="1">
+      <c r="B4" s="109"/>
       <c r="C4" s="24" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="96"/>
+      <c r="F4" s="109"/>
       <c r="G4" s="24" t="s">
         <v>0</v>
       </c>
       <c r="H4" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="96"/>
+      <c r="J4" s="109"/>
       <c r="K4" s="45" t="s">
         <v>0</v>
       </c>
       <c r="L4" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="N4" s="96"/>
+      <c r="N4" s="112"/>
       <c r="O4" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="P4" s="71" t="s">
+      <c r="P4" s="90" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="2:16" ht="24" customHeight="1">
+      <c r="Q4" s="91"/>
+      <c r="R4" s="112"/>
+      <c r="S4" s="93" t="s">
+        <v>0</v>
+      </c>
+      <c r="T4" s="93" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="2:20" ht="24" customHeight="1">
       <c r="B5" s="4">
         <v>45992</v>
       </c>
@@ -5521,8 +5726,17 @@
       <c r="P5" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="6" spans="2:16" ht="24" customHeight="1">
+      <c r="R5" s="4">
+        <v>46114</v>
+      </c>
+      <c r="S5" s="95" t="s">
+        <v>5</v>
+      </c>
+      <c r="T5" s="25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="2:20" ht="24" customHeight="1">
       <c r="B6" s="4">
         <v>45993</v>
       </c>
@@ -5557,8 +5771,17 @@
       <c r="P6" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="7" spans="2:16" ht="24" customHeight="1">
+      <c r="R6" s="4">
+        <v>46115</v>
+      </c>
+      <c r="S6" s="96" t="s">
+        <v>5</v>
+      </c>
+      <c r="T6" s="25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20" ht="24" customHeight="1">
       <c r="B7" s="4">
         <v>45994</v>
       </c>
@@ -5593,8 +5816,17 @@
       <c r="P7" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="8" spans="2:16" ht="24" customHeight="1">
+      <c r="R7" s="4">
+        <v>46116</v>
+      </c>
+      <c r="S7" s="99" t="s">
+        <v>33</v>
+      </c>
+      <c r="T7" s="99" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="2:20" ht="24" customHeight="1">
       <c r="B8" s="4">
         <v>45995</v>
       </c>
@@ -5632,8 +5864,17 @@
       <c r="P8" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="9" spans="2:16" ht="24" customHeight="1">
+      <c r="R8" s="4">
+        <v>46117</v>
+      </c>
+      <c r="S8" s="101" t="s">
+        <v>5</v>
+      </c>
+      <c r="T8" s="25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20" ht="24" customHeight="1">
       <c r="B9" s="4">
         <v>45996</v>
       </c>
@@ -5671,8 +5912,17 @@
       <c r="P9" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="10" spans="2:16" ht="24" customHeight="1">
+      <c r="R9" s="4">
+        <v>46118</v>
+      </c>
+      <c r="S9" s="83" t="s">
+        <v>32</v>
+      </c>
+      <c r="T9" s="83">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" ht="24" customHeight="1">
       <c r="B10" s="4">
         <v>45997</v>
       </c>
@@ -5710,8 +5960,17 @@
       <c r="P10" s="76" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="11" spans="2:16" ht="24" customHeight="1">
+      <c r="R10" s="4">
+        <v>46119</v>
+      </c>
+      <c r="S10" s="83" t="s">
+        <v>32</v>
+      </c>
+      <c r="T10" s="83">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" ht="24" customHeight="1">
       <c r="B11" s="4">
         <v>45998</v>
       </c>
@@ -5749,8 +6008,17 @@
       <c r="P11" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="12" spans="2:16" ht="24" customHeight="1">
+      <c r="R11" s="4">
+        <v>46120</v>
+      </c>
+      <c r="S11" s="83" t="s">
+        <v>32</v>
+      </c>
+      <c r="T11" s="83">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20" ht="24" customHeight="1">
       <c r="B12" s="4">
         <v>45999</v>
       </c>
@@ -5788,8 +6056,9 @@
       <c r="P12" s="77">
         <v>100</v>
       </c>
-    </row>
-    <row r="13" spans="2:16" ht="24" customHeight="1">
+      <c r="R12" s="91"/>
+    </row>
+    <row r="13" spans="2:20" ht="24" customHeight="1">
       <c r="B13" s="4">
         <v>46000</v>
       </c>
@@ -5827,8 +6096,9 @@
       <c r="P13" s="77">
         <v>100</v>
       </c>
-    </row>
-    <row r="14" spans="2:16" ht="24" customHeight="1">
+      <c r="R13" s="91"/>
+    </row>
+    <row r="14" spans="2:20" ht="24" customHeight="1">
       <c r="B14" s="4">
         <v>46001</v>
       </c>
@@ -5866,8 +6136,9 @@
       <c r="P14" s="77" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="15" spans="2:16" ht="24" customHeight="1">
+      <c r="R14" s="91"/>
+    </row>
+    <row r="15" spans="2:20" ht="24" customHeight="1">
       <c r="B15" s="4">
         <v>46002</v>
       </c>
@@ -5905,8 +6176,9 @@
       <c r="P15" s="77" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="16" spans="2:16" ht="24" customHeight="1">
+      <c r="R15" s="91"/>
+    </row>
+    <row r="16" spans="2:20" ht="24" customHeight="1">
       <c r="B16" s="4">
         <v>46003</v>
       </c>
@@ -5944,8 +6216,9 @@
       <c r="P16" s="77" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="17" spans="2:17" ht="24" customHeight="1">
+      <c r="R16" s="91"/>
+    </row>
+    <row r="17" spans="2:18" ht="24" customHeight="1">
       <c r="B17" s="4">
         <v>46004</v>
       </c>
@@ -5983,8 +6256,9 @@
       <c r="P17" s="78" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="18" spans="2:17" ht="24" customHeight="1">
+      <c r="R17" s="91"/>
+    </row>
+    <row r="18" spans="2:18" ht="24" customHeight="1">
       <c r="B18" s="4">
         <v>46005</v>
       </c>
@@ -6022,8 +6296,9 @@
       <c r="P18" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="19" spans="2:17" ht="24" customHeight="1">
+      <c r="R18" s="91"/>
+    </row>
+    <row r="19" spans="2:18" ht="24" customHeight="1">
       <c r="B19" s="4">
         <v>46006</v>
       </c>
@@ -6061,8 +6336,9 @@
       <c r="P19" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="20" spans="2:17" ht="24" customHeight="1">
+      <c r="R19" s="91"/>
+    </row>
+    <row r="20" spans="2:18" ht="24" customHeight="1">
       <c r="B20" s="4">
         <v>46007</v>
       </c>
@@ -6100,8 +6376,9 @@
       <c r="P20" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="21" spans="2:17" ht="24" customHeight="1">
+      <c r="R20" s="91"/>
+    </row>
+    <row r="21" spans="2:18" ht="24" customHeight="1">
       <c r="B21" s="4">
         <v>46008</v>
       </c>
@@ -6139,8 +6416,9 @@
       <c r="P21" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="22" spans="2:17" ht="24" customHeight="1">
+      <c r="R21" s="91"/>
+    </row>
+    <row r="22" spans="2:18" ht="24" customHeight="1">
       <c r="B22" s="4">
         <v>46009</v>
       </c>
@@ -6178,8 +6456,9 @@
       <c r="P22" s="80">
         <v>100</v>
       </c>
-    </row>
-    <row r="23" spans="2:17" ht="24" customHeight="1">
+      <c r="R22" s="91"/>
+    </row>
+    <row r="23" spans="2:18" ht="24" customHeight="1">
       <c r="B23" s="4">
         <v>46010</v>
       </c>
@@ -6217,8 +6496,9 @@
       <c r="P23" s="80">
         <v>100</v>
       </c>
-    </row>
-    <row r="24" spans="2:17" ht="24" customHeight="1">
+      <c r="R23" s="91"/>
+    </row>
+    <row r="24" spans="2:18" ht="24" customHeight="1">
       <c r="B24" s="4">
         <v>46011</v>
       </c>
@@ -6256,8 +6536,9 @@
       <c r="P24" s="81" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="25" spans="2:17" ht="24" customHeight="1">
+      <c r="R24" s="91"/>
+    </row>
+    <row r="25" spans="2:18" ht="24" customHeight="1">
       <c r="B25" s="4">
         <v>46012</v>
       </c>
@@ -6295,8 +6576,9 @@
       <c r="P25" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="26" spans="2:17" ht="24" customHeight="1">
+      <c r="R25" s="91"/>
+    </row>
+    <row r="26" spans="2:18" ht="24" customHeight="1">
       <c r="B26" s="4">
         <v>46013</v>
       </c>
@@ -6329,16 +6611,15 @@
         <v>46104</v>
       </c>
       <c r="O26" s="83" t="s">
-        <v>28</v>
-      </c>
-      <c r="P26" s="83" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q26" s="83">
-        <v>-350</v>
-      </c>
-    </row>
-    <row r="27" spans="2:17" ht="24" customHeight="1">
+        <v>32</v>
+      </c>
+      <c r="P26" s="83">
+        <v>350</v>
+      </c>
+      <c r="Q26" s="83"/>
+      <c r="R26" s="91"/>
+    </row>
+    <row r="27" spans="2:18" ht="24" customHeight="1">
       <c r="B27" s="4">
         <v>46014</v>
       </c>
@@ -6376,8 +6657,9 @@
       <c r="P27" s="82">
         <v>100</v>
       </c>
-    </row>
-    <row r="28" spans="2:17" ht="24" customHeight="1">
+      <c r="R27" s="91"/>
+    </row>
+    <row r="28" spans="2:18" ht="24" customHeight="1">
       <c r="B28" s="4">
         <v>46015</v>
       </c>
@@ -6415,8 +6697,9 @@
       <c r="P28" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="29" spans="2:17" ht="24" customHeight="1">
+      <c r="R28" s="91"/>
+    </row>
+    <row r="29" spans="2:18" ht="24" customHeight="1">
       <c r="B29" s="4">
         <v>46016</v>
       </c>
@@ -6454,8 +6737,9 @@
       <c r="P29" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="30" spans="2:17" ht="24" customHeight="1">
+      <c r="R29" s="91"/>
+    </row>
+    <row r="30" spans="2:18" ht="24" customHeight="1">
       <c r="B30" s="4">
         <v>46017</v>
       </c>
@@ -6493,8 +6777,9 @@
       <c r="P30" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="31" spans="2:17" ht="24" customHeight="1">
+      <c r="R30" s="91"/>
+    </row>
+    <row r="31" spans="2:18" ht="24" customHeight="1">
       <c r="B31" s="4">
         <v>46018</v>
       </c>
@@ -6532,8 +6817,9 @@
       <c r="P31" s="86" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="32" spans="2:17" ht="24" customHeight="1">
+      <c r="R31" s="91"/>
+    </row>
+    <row r="32" spans="2:18" ht="24" customHeight="1">
       <c r="B32" s="4">
         <v>46019</v>
       </c>
@@ -6567,8 +6853,9 @@
       <c r="P32" s="25">
         <v>100</v>
       </c>
-    </row>
-    <row r="33" spans="2:8" ht="24" customHeight="1">
+      <c r="R32" s="91"/>
+    </row>
+    <row r="33" spans="2:18" ht="24" customHeight="1">
       <c r="B33" s="4">
         <v>46020</v>
       </c>
@@ -6587,8 +6874,18 @@
       <c r="H33" s="44" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="34" spans="2:8" ht="24" customHeight="1">
+      <c r="N33" s="4">
+        <v>46111</v>
+      </c>
+      <c r="O33" s="91" t="s">
+        <v>5</v>
+      </c>
+      <c r="P33" s="91">
+        <v>100</v>
+      </c>
+      <c r="R33" s="91"/>
+    </row>
+    <row r="34" spans="2:18" ht="24" customHeight="1">
       <c r="B34" s="4">
         <v>46021</v>
       </c>
@@ -6607,8 +6904,18 @@
       <c r="H34" s="44">
         <v>100</v>
       </c>
-    </row>
-    <row r="35" spans="2:8" ht="24" customHeight="1">
+      <c r="N34" s="4">
+        <v>46112</v>
+      </c>
+      <c r="O34" s="91" t="s">
+        <v>5</v>
+      </c>
+      <c r="P34" s="91">
+        <v>100</v>
+      </c>
+      <c r="R34" s="91"/>
+    </row>
+    <row r="35" spans="2:18" ht="24" customHeight="1">
       <c r="B35" s="4">
         <v>46022</v>
       </c>
@@ -6627,8 +6934,12 @@
       <c r="H35" s="44">
         <v>100</v>
       </c>
-    </row>
-    <row r="36" spans="2:8" ht="24" customHeight="1">
+      <c r="N35" s="4">
+        <v>46113</v>
+      </c>
+      <c r="R35" s="91"/>
+    </row>
+    <row r="36" spans="2:18" ht="24" customHeight="1">
       <c r="B36" s="4">
         <v>46023</v>
       </c>
@@ -6647,8 +6958,15 @@
       <c r="H36" s="25">
         <v>7800</v>
       </c>
-    </row>
-    <row r="37" spans="2:8" ht="24" customHeight="1">
+      <c r="N36" s="4">
+        <v>46114</v>
+      </c>
+      <c r="O36" s="95"/>
+      <c r="P36" s="25">
+        <v>7950</v>
+      </c>
+    </row>
+    <row r="37" spans="2:18" ht="24" customHeight="1">
       <c r="B37" s="4">
         <v>46024</v>
       </c>
@@ -6659,7 +6977,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="2:8" ht="24" customHeight="1">
+    <row r="38" spans="2:18" ht="24" customHeight="1">
       <c r="B38" s="4">
         <v>46025</v>
       </c>
@@ -6671,15 +6989,17 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="N2:N4"/>
-    <mergeCell ref="O2:P3"/>
-    <mergeCell ref="K2:L3"/>
+  <mergeCells count="10">
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="C2:D3"/>
     <mergeCell ref="F2:F4"/>
     <mergeCell ref="G2:H3"/>
     <mergeCell ref="J2:J4"/>
+    <mergeCell ref="R2:R4"/>
+    <mergeCell ref="S2:T3"/>
+    <mergeCell ref="N2:N4"/>
+    <mergeCell ref="O2:P3"/>
+    <mergeCell ref="K2:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6688,85 +7008,103 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:Q36"/>
+  <dimension ref="A2:U36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.5703125" defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="16384" width="17.5703125" style="29"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:17" ht="24" customHeight="1">
-      <c r="B2" s="96"/>
-      <c r="C2" s="90">
+    <row r="2" spans="1:21" ht="24" customHeight="1">
+      <c r="B2" s="109"/>
+      <c r="C2" s="103">
         <f>SUM(D5:D44)</f>
         <v>10500</v>
       </c>
-      <c r="D2" s="90"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="90">
+      <c r="D2" s="103"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="103">
         <f>SUM(H5:H44)</f>
         <v>10500</v>
       </c>
-      <c r="H2" s="90"/>
-      <c r="K2" s="96"/>
-      <c r="L2" s="90">
+      <c r="H2" s="103"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="103">
         <f>SUM(M5:M37)</f>
         <v>5250</v>
       </c>
-      <c r="M2" s="90"/>
-      <c r="O2" s="96">
+      <c r="M2" s="103"/>
+      <c r="O2" s="109">
         <v>3</v>
       </c>
-      <c r="P2" s="90">
+      <c r="P2" s="103">
         <f>SUM(Q5:Q37)</f>
-        <v>360</v>
-      </c>
-      <c r="Q2" s="90"/>
-    </row>
-    <row r="3" spans="1:17" ht="24" customHeight="1">
-      <c r="B3" s="96"/>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="K3" s="96"/>
-      <c r="L3" s="90"/>
-      <c r="M3" s="90"/>
-      <c r="O3" s="96"/>
-      <c r="P3" s="90"/>
-      <c r="Q3" s="90"/>
-    </row>
-    <row r="4" spans="1:17" ht="24" customHeight="1">
-      <c r="B4" s="96"/>
+        <v>10500</v>
+      </c>
+      <c r="Q2" s="103"/>
+      <c r="S2" s="109">
+        <v>4</v>
+      </c>
+      <c r="T2" s="103">
+        <f>SUM(U5:U37)</f>
+        <v>530</v>
+      </c>
+      <c r="U2" s="103"/>
+    </row>
+    <row r="3" spans="1:21" ht="24" customHeight="1">
+      <c r="B3" s="109"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="F3" s="109"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
+      <c r="K3" s="109"/>
+      <c r="L3" s="103"/>
+      <c r="M3" s="103"/>
+      <c r="O3" s="109"/>
+      <c r="P3" s="103"/>
+      <c r="Q3" s="103"/>
+      <c r="S3" s="109"/>
+      <c r="T3" s="103"/>
+      <c r="U3" s="103"/>
+    </row>
+    <row r="4" spans="1:21" ht="24" customHeight="1">
+      <c r="B4" s="109"/>
       <c r="C4" s="28" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="96"/>
+      <c r="F4" s="109"/>
       <c r="G4" s="33" t="s">
         <v>0</v>
       </c>
       <c r="H4" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="K4" s="96"/>
+      <c r="K4" s="109"/>
       <c r="L4" s="57" t="s">
         <v>0</v>
       </c>
       <c r="M4" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="O4" s="96"/>
+      <c r="O4" s="109"/>
       <c r="P4" s="71" t="s">
         <v>0</v>
       </c>
       <c r="Q4" s="71" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" ht="24" customHeight="1">
+      <c r="S4" s="109"/>
+      <c r="T4" s="93" t="s">
+        <v>0</v>
+      </c>
+      <c r="U4" s="93" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" ht="24" customHeight="1">
       <c r="B5" s="31">
         <v>46006</v>
       </c>
@@ -6803,8 +7141,17 @@
       <c r="Q5" s="72" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" ht="24" customHeight="1">
+      <c r="S5" s="4">
+        <v>46114</v>
+      </c>
+      <c r="T5" s="95" t="s">
+        <v>5</v>
+      </c>
+      <c r="U5" s="29">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" ht="24" customHeight="1">
       <c r="A6" s="30"/>
       <c r="B6" s="31">
         <v>46007</v>
@@ -6843,8 +7190,17 @@
       <c r="Q6" s="29">
         <v>60</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="24" customHeight="1">
+      <c r="S6" s="4">
+        <v>46115</v>
+      </c>
+      <c r="T6" s="96" t="s">
+        <v>33</v>
+      </c>
+      <c r="U6" s="96" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" ht="24" customHeight="1">
       <c r="A7" s="30"/>
       <c r="B7" s="31">
         <v>46008</v>
@@ -6883,8 +7239,17 @@
       <c r="Q7" s="82">
         <v>60</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="24" customHeight="1">
+      <c r="S7" s="4">
+        <v>46116</v>
+      </c>
+      <c r="T7" s="83" t="s">
+        <v>32</v>
+      </c>
+      <c r="U7" s="83">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" ht="24" customHeight="1">
       <c r="A8" s="30"/>
       <c r="B8" s="31">
         <v>46009</v>
@@ -6923,8 +7288,17 @@
       <c r="Q8" s="82">
         <v>60</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" ht="24" customHeight="1">
+      <c r="S8" s="4">
+        <v>46117</v>
+      </c>
+      <c r="T8" s="100" t="s">
+        <v>5</v>
+      </c>
+      <c r="U8" s="29">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" ht="24" customHeight="1">
       <c r="A9" s="30"/>
       <c r="B9" s="31">
         <v>46010</v>
@@ -6963,8 +7337,17 @@
       <c r="Q9" s="75">
         <v>60</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" ht="24" customHeight="1">
+      <c r="S9" s="4">
+        <v>46118</v>
+      </c>
+      <c r="T9" s="101" t="s">
+        <v>5</v>
+      </c>
+      <c r="U9" s="101">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" ht="24" customHeight="1">
       <c r="A10" s="30"/>
       <c r="B10" s="31">
         <v>46011</v>
@@ -7004,7 +7387,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="24" customHeight="1">
+    <row r="11" spans="1:21" ht="24" customHeight="1">
       <c r="A11" s="30"/>
       <c r="B11" s="31">
         <v>46012</v>
@@ -7044,7 +7427,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="24" customHeight="1">
+    <row r="12" spans="1:21" ht="24" customHeight="1">
       <c r="A12" s="30"/>
       <c r="B12" s="31">
         <v>46013</v>
@@ -7084,7 +7467,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="24" customHeight="1">
+    <row r="13" spans="1:21" ht="24" customHeight="1">
       <c r="A13" s="30"/>
       <c r="B13" s="31">
         <v>46014</v>
@@ -7114,11 +7497,17 @@
         <v>60</v>
       </c>
       <c r="N13" s="70"/>
-      <c r="O13" s="4"/>
-      <c r="P13" s="77"/>
-      <c r="Q13" s="77"/>
-    </row>
-    <row r="14" spans="1:17" ht="24" customHeight="1">
+      <c r="O13" s="4">
+        <v>46111</v>
+      </c>
+      <c r="P13" s="89" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q13" s="77">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" ht="24" customHeight="1">
       <c r="A14" s="30"/>
       <c r="B14" s="31">
         <v>46015</v>
@@ -7148,11 +7537,17 @@
         <v>60</v>
       </c>
       <c r="N14" s="70"/>
-      <c r="O14" s="4"/>
-      <c r="P14" s="77"/>
-      <c r="Q14" s="77"/>
-    </row>
-    <row r="15" spans="1:17" ht="24" customHeight="1">
+      <c r="O14" s="4">
+        <v>46112</v>
+      </c>
+      <c r="P14" s="91" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q14" s="77">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" ht="24" customHeight="1">
       <c r="A15" s="30"/>
       <c r="B15" s="31">
         <v>46016</v>
@@ -7182,11 +7577,17 @@
         <v>60</v>
       </c>
       <c r="N15" s="70"/>
-      <c r="O15" s="4"/>
-      <c r="P15" s="77"/>
-      <c r="Q15" s="77"/>
-    </row>
-    <row r="16" spans="1:17" ht="24" customHeight="1">
+      <c r="O15" s="4">
+        <v>46113</v>
+      </c>
+      <c r="P15" s="91" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q15" s="77">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" ht="24" customHeight="1">
       <c r="A16" s="30"/>
       <c r="B16" s="31">
         <v>46017</v>
@@ -7216,9 +7617,15 @@
         <v>28</v>
       </c>
       <c r="N16" s="70"/>
-      <c r="O16" s="4"/>
-      <c r="P16" s="77"/>
-      <c r="Q16" s="77"/>
+      <c r="O16" s="4">
+        <v>46114</v>
+      </c>
+      <c r="P16" s="92" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q16" s="77">
+        <v>9960</v>
+      </c>
     </row>
     <row r="17" spans="1:17" ht="21">
       <c r="A17" s="30"/>
@@ -7363,7 +7770,7 @@
       <c r="H21" s="44">
         <v>60</v>
       </c>
-      <c r="I21" s="97"/>
+      <c r="I21" s="113"/>
     </row>
     <row r="22" spans="1:17" ht="21">
       <c r="A22" s="30"/>
@@ -7385,7 +7792,7 @@
       <c r="H22" s="44">
         <v>60</v>
       </c>
-      <c r="I22" s="97"/>
+      <c r="I22" s="113"/>
     </row>
     <row r="23" spans="1:17" ht="21">
       <c r="A23" s="30"/>
@@ -7681,16 +8088,18 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="O2:O4"/>
-    <mergeCell ref="P2:Q3"/>
-    <mergeCell ref="L2:M3"/>
+  <mergeCells count="11">
+    <mergeCell ref="K2:K4"/>
     <mergeCell ref="I21:I22"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="C2:D3"/>
     <mergeCell ref="F2:F4"/>
     <mergeCell ref="G2:H3"/>
-    <mergeCell ref="K2:K4"/>
+    <mergeCell ref="S2:S4"/>
+    <mergeCell ref="T2:U3"/>
+    <mergeCell ref="O2:O4"/>
+    <mergeCell ref="P2:Q3"/>
+    <mergeCell ref="L2:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>